<commit_message>
Recount module completion; regrade three AI-governance rows
The dashboard still carried pre-AI-governance numbers while the Platform tab
had already been rewritten, so the workbook disagreed with itself: 43.6% on
one sheet, 59% on the other. Every module is now recounted from its own rows.

Three Platform features drop from Done to Partial. lib/ai/policy.ts,
lib/ai/budget.ts and the ai_usage_ledger table have code and live schema, but
nothing imports them and the ledger has no INSERT site anywhere in src/ - the
same condition on which the response cache was already graded Partial. A
policy nothing consults and a budget nothing checks do not constrain anything.

Platform / Core 43.6% -> 55.0%, total 47.7% -> 51.1% across 132 features.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Preckon-system/Preckon_Module_Completion.xlsx
+++ b/Preckon-system/Preckon_Module_Completion.xlsx
@@ -29,8 +29,8 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'ScheduleLogix'!$A$4:$G$19</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'ProcureLogix'!$A$4:$G$10</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'NarrativeLogix'!$A$4:$G$7</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'Platform-Core'!$A$4:$G$43</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'P0 Backlog'!$A$4:$F$22</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'Platform-Core'!$A$4:$G$44</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'P0 Backlog'!$A$4:$F$20</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -288,7 +288,6 @@
 
 <file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
 <chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
-  <style val="10"/>
   <chart>
     <title>
       <tx>
@@ -724,10 +723,11 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Every feature verified against the codebase and the deployed database on 20 Aug 2026. Weighted: Done 1.0, Partial 0.5, Scaffolded 0.25, Missing 0.</t>
-        </is>
-      </c>
-    </row>
+          <t>Every feature verified against the codebase and the deployed database on 20 Aug 2026, after the 13:00 deploy (app and worker rebuilt, all 21 migrations applied, DocLogix and AI-governance tables live). Weighted: Done 1.0, Partial 0.5, Scaffolded 0.25, Missing 0. This revision recounts every module from its own rows and regrades three AI-governance features from Done to Partial - policy, budgets and the usage ledger have code and tables but no caller, which is the same basis on which the cache was already Partial.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3"/>
     <row r="4" ht="34" customHeight="1">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -1083,31 +1083,32 @@
         </is>
       </c>
       <c r="C13" s="6" t="n">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="D13" s="6" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="E13" s="6" t="n">
-        <v>4</v>
+        <v>12</v>
       </c>
       <c r="F13" s="6" t="n">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="G13" s="7" t="n">
-        <v>0.436</v>
+        <v>0.55</v>
       </c>
       <c r="H13" s="8" t="inlineStr">
         <is>
-          <t>█████████░░░░░░░░░░░</t>
+          <t>███████████░░░░░░░░░</t>
         </is>
       </c>
       <c r="I13" s="5" t="inlineStr">
         <is>
-          <t>Trust foundations are strong: audit chain, tenant isolation, durable jobs, provenance. AI governance and enterprise ops are the gaps.</t>
-        </is>
-      </c>
-    </row>
+          <t>Trust foundations are strong: audit chain, tenant isolation, durable jobs, provenance. The AI governance layer landed on 20 Aug - policy, model registry, prompt versions, budgets, cache and usage ledger all have code and live tables - but nothing imports any of it yet, so it is graded Partial: built, not yet enforced. Enterprise ops remain the real gap.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14"/>
     <row r="15" ht="40" customHeight="1">
       <c r="A15" s="11" t="inlineStr">
         <is>
@@ -1120,19 +1121,19 @@
         </is>
       </c>
       <c r="C15" s="12" t="n">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="D15" s="12" t="n">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="E15" s="12" t="n">
-        <v>23</v>
+        <v>31</v>
       </c>
       <c r="F15" s="12" t="n">
-        <v>57</v>
+        <v>49</v>
       </c>
       <c r="G15" s="13" t="n">
-        <v>0.477</v>
+        <v>0.511</v>
       </c>
       <c r="H15" s="14" t="inlineStr">
         <is>
@@ -1161,7 +1162,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G43"/>
+  <dimension ref="A1:G44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -1176,17 +1177,18 @@
     <row r="1" ht="24" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Platform / Core - 44% complete</t>
+          <t>Platform / Core - 55% complete</t>
         </is>
       </c>
     </row>
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Identity, tenancy, audit, AI governance, operations.  39 features audited: 15 done, 4 partial, 20 missing.</t>
-        </is>
-      </c>
-    </row>
+          <t>Identity, tenancy, audit, AI governance, operations.  40 features audited: 19 done, 9 partial, 12 missing.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3"/>
     <row r="4" ht="34" customHeight="1">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -1642,19 +1644,19 @@
           <t>Per-attempt usage ledger</t>
         </is>
       </c>
-      <c r="C16" s="17" t="inlineStr">
-        <is>
-          <t>Missing</t>
+      <c r="C16" s="16" t="inlineStr">
+        <is>
+          <t>Partial</t>
         </is>
       </c>
       <c r="D16" s="5" t="inlineStr">
         <is>
-          <t>ai_job holds one MUTABLE row per job.</t>
+          <t>ai_usage_ledger - append-only, one row per attempt, with model alias, prompt version, sensitivity, policy version, cost and outcome. Migration 021.</t>
         </is>
       </c>
       <c r="E16" s="5" t="inlineStr">
         <is>
-          <t>A retry overwrites the previous attempt tokens, so failed-attempt spend is invisible and AI cost is under-counted today.</t>
+          <t>No writer: ai_usage_ledger has no INSERT site in src/. Table is live; nothing records to it.</t>
         </is>
       </c>
       <c r="F16" s="17" t="inlineStr">
@@ -1679,19 +1681,19 @@
           <t>Tenant AI policy and data sensitivity</t>
         </is>
       </c>
-      <c r="C17" s="17" t="inlineStr">
-        <is>
-          <t>Missing</t>
+      <c r="C17" s="16" t="inlineStr">
+        <is>
+          <t>Partial</t>
         </is>
       </c>
       <c r="D17" s="5" t="inlineStr">
         <is>
-          <t>No sensitivity field anywhere in src.</t>
+          <t>ai/policy.ts + ai_tenant_policy - deployment modes, per-classification boundaries, eligibility before scoring, tenant may narrow never widen. 47 tests.</t>
         </is>
       </c>
       <c r="E17" s="5" t="inlineStr">
         <is>
-          <t>Blocks Preckon Private AI and Sovereign AI as sellable products.</t>
+          <t>Not imported by any file. Policy that nothing consults does not constrain anything.</t>
         </is>
       </c>
       <c r="F17" s="17" t="inlineStr">
@@ -1716,19 +1718,19 @@
           <t>Model registry and aliases</t>
         </is>
       </c>
-      <c r="C18" s="17" t="inlineStr">
-        <is>
-          <t>Missing</t>
+      <c r="C18" s="18" t="inlineStr">
+        <is>
+          <t>Partial</t>
         </is>
       </c>
       <c r="D18" s="5" t="inlineStr">
         <is>
-          <t>Model names hard-coded in 3 routes and jobs.ts.</t>
+          <t>ai/registry.ts + ai_model_registry - aliases, capabilities, rate cards, loud failure on unknown alias. 37 tests with cache.</t>
         </is>
       </c>
       <c r="E18" s="5" t="inlineStr">
         <is>
-          <t>Application code must reference aliases, not claude-opus-4-8.</t>
+          <t>The four files naming concrete models are not yet migrated to aliases.</t>
         </is>
       </c>
       <c r="F18" s="18" t="inlineStr">
@@ -1753,19 +1755,19 @@
           <t>Prompt registry with versions</t>
         </is>
       </c>
-      <c r="C19" s="17" t="inlineStr">
-        <is>
-          <t>Missing</t>
+      <c r="C19" s="18" t="inlineStr">
+        <is>
+          <t>Partial</t>
         </is>
       </c>
       <c r="D19" s="5" t="inlineStr">
         <is>
-          <t>Prompts are strings in worker/src/prompts.mjs.</t>
+          <t>ai_prompt_version table with prompt_key, version, task_type, prefix hash and approval status.</t>
         </is>
       </c>
       <c r="E19" s="5" t="inlineStr">
         <is>
-          <t>AI Fabric section 18 forbids untracked prompt strings in source.</t>
+          <t>The worker still reads its prompts from source; nothing populates the table yet.</t>
         </is>
       </c>
       <c r="F19" s="18" t="inlineStr">
@@ -1790,19 +1792,19 @@
           <t>Budgets (token, cost, latency)</t>
         </is>
       </c>
-      <c r="C20" s="17" t="inlineStr">
-        <is>
-          <t>Missing</t>
+      <c r="C20" s="16" t="inlineStr">
+        <is>
+          <t>Partial</t>
         </is>
       </c>
       <c r="D20" s="5" t="inlineStr">
         <is>
-          <t>None.</t>
+          <t>ai/budget.ts - estimate before running, tenant limits, clamping, remedies in the order section 21 recommends. 47 tests with policy.</t>
         </is>
       </c>
       <c r="E20" s="5" t="inlineStr">
         <is>
-          <t>Router must reject or re-route when a budget would be exceeded.</t>
+          <t>Not imported by any file. A budget nothing checks caps nothing.</t>
         </is>
       </c>
       <c r="F20" s="18" t="inlineStr">
@@ -1827,19 +1829,19 @@
           <t>Response cache (exact, semantic, artifact)</t>
         </is>
       </c>
-      <c r="C21" s="17" t="inlineStr">
-        <is>
-          <t>Missing</t>
+      <c r="C21" s="18" t="inlineStr">
+        <is>
+          <t>Partial</t>
         </is>
       </c>
       <c r="D21" s="5" t="inlineStr">
         <is>
-          <t>None.</t>
+          <t>ai/cache.ts + ai_response_cache - every answer-changing dimension in the key, scoped invalidation triggers. 37 tests.</t>
         </is>
       </c>
       <c r="E21" s="5" t="inlineStr">
         <is>
-          <t>No cache layer of any kind.</t>
+          <t>Keys and safety rules exist; nothing reads or writes the table yet.</t>
         </is>
       </c>
       <c r="F21" s="18" t="inlineStr">
@@ -2209,7 +2211,7 @@
       </c>
       <c r="E31" s="5" t="inlineStr">
         <is>
-          <t>426 tests and six quality gates run only on a developer machine.</t>
+          <t>426 tests and six quality gates run only on a developer machine. The publishing token also lacks `workflow` scope, so ci.yml cannot even be pushed to techsmeinc/preckon-tenant - the mirror carries no .github at all.</t>
         </is>
       </c>
       <c r="F31" s="17" t="inlineStr">
@@ -2342,7 +2344,7 @@
       </c>
       <c r="B35" s="5" t="inlineStr">
         <is>
-          <t>Repeatable deploy</t>
+          <t>schema.sql / migration drift guard</t>
         </is>
       </c>
       <c r="C35" s="16" t="inlineStr">
@@ -2352,7 +2354,7 @@
       </c>
       <c r="D35" s="5" t="inlineStr">
         <is>
-          <t>deploy.ps1 - sha256-verified resumable upload, migrations, catalog seed gate, worker rebuild.</t>
+          <t>schema-drift.test.ts - fails if a migration creates a table schema.sql does not declare. Found 5 tables drifted since migration 004 whose queries had never been tenant-checked.</t>
         </is>
       </c>
       <c r="E35" s="5" t="inlineStr">
@@ -2374,27 +2376,27 @@
     <row r="36">
       <c r="A36" s="15" t="inlineStr">
         <is>
-          <t>Security</t>
+          <t>Ops</t>
         </is>
       </c>
       <c r="B36" s="5" t="inlineStr">
         <is>
-          <t>Encryption at rest and key management</t>
-        </is>
-      </c>
-      <c r="C36" s="17" t="inlineStr">
-        <is>
-          <t>Missing</t>
+          <t>Repeatable deploy</t>
+        </is>
+      </c>
+      <c r="C36" s="16" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="D36" s="5" t="inlineStr">
         <is>
-          <t>None.</t>
+          <t>deploy.ps1 - sha256-verified resumable upload, migrations, catalog seed gate, worker rebuild.</t>
         </is>
       </c>
       <c r="E36" s="5" t="inlineStr">
         <is>
-          <t>Named in Complete Platform section 15.</t>
+          <t>-</t>
         </is>
       </c>
       <c r="F36" s="17" t="inlineStr">
@@ -2404,7 +2406,7 @@
       </c>
       <c r="G36" s="6" t="inlineStr">
         <is>
-          <t>L</t>
+          <t>-</t>
         </is>
       </c>
     </row>
@@ -2416,7 +2418,7 @@
       </c>
       <c r="B37" s="5" t="inlineStr">
         <is>
-          <t>Secrets management (Vault / KMS)</t>
+          <t>Encryption at rest and key management</t>
         </is>
       </c>
       <c r="C37" s="17" t="inlineStr">
@@ -2426,22 +2428,22 @@
       </c>
       <c r="D37" s="5" t="inlineStr">
         <is>
-          <t>Secrets in .env on the host.</t>
+          <t>None.</t>
         </is>
       </c>
       <c r="E37" s="5" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F37" s="18" t="inlineStr">
-        <is>
-          <t>P1</t>
+          <t>Named in Complete Platform section 15.</t>
+        </is>
+      </c>
+      <c r="F37" s="17" t="inlineStr">
+        <is>
+          <t>P0</t>
         </is>
       </c>
       <c r="G37" s="6" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>L</t>
         </is>
       </c>
     </row>
@@ -2453,7 +2455,7 @@
       </c>
       <c r="B38" s="5" t="inlineStr">
         <is>
-          <t>Credential rotation</t>
+          <t>Secrets management (Vault / KMS)</t>
         </is>
       </c>
       <c r="C38" s="17" t="inlineStr">
@@ -2463,22 +2465,22 @@
       </c>
       <c r="D38" s="5" t="inlineStr">
         <is>
-          <t>Outstanding from the earlier security review.</t>
+          <t>Secrets in .env on the host.</t>
         </is>
       </c>
       <c r="E38" s="5" t="inlineStr">
         <is>
-          <t>Rotate everything ever committed; confirm the production DB password is not the default.</t>
-        </is>
-      </c>
-      <c r="F38" s="17" t="inlineStr">
-        <is>
-          <t>P0</t>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F38" s="18" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="G38" s="6" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>M</t>
         </is>
       </c>
     </row>
@@ -2490,7 +2492,7 @@
       </c>
       <c r="B39" s="5" t="inlineStr">
         <is>
-          <t>Upload malware scanning</t>
+          <t>Credential rotation</t>
         </is>
       </c>
       <c r="C39" s="17" t="inlineStr">
@@ -2500,22 +2502,22 @@
       </c>
       <c r="D39" s="5" t="inlineStr">
         <is>
-          <t>None.</t>
+          <t>Outstanding from the earlier security review.</t>
         </is>
       </c>
       <c r="E39" s="5" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F39" s="18" t="inlineStr">
-        <is>
-          <t>P1</t>
+          <t>Rotate everything ever committed; confirm the production DB password is not the default.</t>
+        </is>
+      </c>
+      <c r="F39" s="17" t="inlineStr">
+        <is>
+          <t>P0</t>
         </is>
       </c>
       <c r="G39" s="6" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>S</t>
         </is>
       </c>
     </row>
@@ -2527,7 +2529,7 @@
       </c>
       <c r="B40" s="5" t="inlineStr">
         <is>
-          <t>Port hardening</t>
+          <t>Upload validation and scan gating</t>
         </is>
       </c>
       <c r="C40" s="18" t="inlineStr">
@@ -2537,138 +2539,175 @@
       </c>
       <c r="D40" s="5" t="inlineStr">
         <is>
-          <t>3308, 4000 and 8081 bind to 127.0.0.1 and are externally closed.</t>
+          <t>upload-safety.ts - magic-number vs extension, blocked extensions, macro formats, path traversal, zip-bomb ratio, explicit scan states. 33 tests.</t>
         </is>
       </c>
       <c r="E40" s="5" t="inlineStr">
         <is>
-          <t>3307 (MySQL), 11434 (Ollama, unauthenticated) and 5000 bind 0.0.0.0; only the provider firewall stops them.</t>
-        </is>
-      </c>
-      <c r="F40" s="17" t="inlineStr">
-        <is>
-          <t>P0</t>
+          <t>Explicitly not an antivirus. A real scanner still needs to sit behind it, and the upload route does not call this yet.</t>
+        </is>
+      </c>
+      <c r="F40" s="18" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="G40" s="6" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>M</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="15" t="inlineStr">
         <is>
-          <t>Governance</t>
+          <t>Security</t>
         </is>
       </c>
       <c r="B41" s="5" t="inlineStr">
         <is>
-          <t>Architecture Decision Records</t>
-        </is>
-      </c>
-      <c r="C41" s="17" t="inlineStr">
-        <is>
-          <t>Missing</t>
+          <t>Port hardening</t>
+        </is>
+      </c>
+      <c r="C41" s="18" t="inlineStr">
+        <is>
+          <t>Partial</t>
         </is>
       </c>
       <c r="D41" s="5" t="inlineStr">
         <is>
-          <t>No docs/adr directory.</t>
+          <t>3308, 4000 and 8081 bind to 127.0.0.1 and are externally closed.</t>
         </is>
       </c>
       <c r="E41" s="5" t="inlineStr">
         <is>
-          <t>50 ADRs are specified across three blueprints. Zero exist.</t>
-        </is>
-      </c>
-      <c r="F41" s="18" t="inlineStr">
-        <is>
-          <t>P1</t>
+          <t>3307 (MySQL), 11434 (Ollama, unauthenticated) and 5000 bind 0.0.0.0; only the provider firewall stops them.</t>
+        </is>
+      </c>
+      <c r="F41" s="17" t="inlineStr">
+        <is>
+          <t>P0</t>
         </is>
       </c>
       <c r="G41" s="6" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>S</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="15" t="inlineStr">
         <is>
-          <t>Integration</t>
+          <t>Governance</t>
         </is>
       </c>
       <c r="B42" s="5" t="inlineStr">
         <is>
-          <t>Enterprise Integration Hub and connector SDK</t>
-        </is>
-      </c>
-      <c r="C42" s="17" t="inlineStr">
-        <is>
-          <t>Missing</t>
+          <t>Architecture Decision Records</t>
+        </is>
+      </c>
+      <c r="C42" s="18" t="inlineStr">
+        <is>
+          <t>Partial</t>
         </is>
       </c>
       <c r="D42" s="5" t="inlineStr">
         <is>
-          <t>integrations.ts is stub-level.</t>
+          <t>docs/adr - 8 ADRs covering the stack conflict, queue, AI authority, aliases, policy, ledger, cache safety and isolation.</t>
         </is>
       </c>
       <c r="E42" s="5" t="inlineStr">
         <is>
-          <t>No connector runtime, canonical mapping or reconciliation engine.</t>
-        </is>
-      </c>
-      <c r="F42" s="19" t="inlineStr">
-        <is>
-          <t>P2</t>
+          <t>8 of the ~50 specified. The rest are unwritten, but the ones that settle live contradictions are done.</t>
+        </is>
+      </c>
+      <c r="F42" s="18" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="G42" s="6" t="inlineStr">
         <is>
-          <t>XL</t>
+          <t>M</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="15" t="inlineStr">
         <is>
+          <t>Integration</t>
+        </is>
+      </c>
+      <c r="B43" s="5" t="inlineStr">
+        <is>
+          <t>Enterprise Integration Hub and connector SDK</t>
+        </is>
+      </c>
+      <c r="C43" s="17" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="D43" s="5" t="inlineStr">
+        <is>
+          <t>integrations.ts is stub-level.</t>
+        </is>
+      </c>
+      <c r="E43" s="5" t="inlineStr">
+        <is>
+          <t>No connector runtime, canonical mapping or reconciliation engine.</t>
+        </is>
+      </c>
+      <c r="F43" s="19" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="G43" s="6" t="inlineStr">
+        <is>
+          <t>XL</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="15" t="inlineStr">
+        <is>
           <t>Knowledge</t>
         </is>
       </c>
-      <c r="B43" s="5" t="inlineStr">
+      <c r="B44" s="5" t="inlineStr">
         <is>
           <t>Cross-module knowledge graph</t>
         </is>
       </c>
-      <c r="C43" s="18" t="inlineStr">
+      <c r="C44" s="18" t="inlineStr">
         <is>
           <t>Partial</t>
         </is>
       </c>
-      <c r="D43" s="5" t="inlineStr">
+      <c r="D44" s="5" t="inlineStr">
         <is>
           <t>pcm_relationship with typed edges, source and confidence.</t>
         </is>
       </c>
-      <c r="E43" s="5" t="inlineStr">
+      <c r="E44" s="5" t="inlineStr">
         <is>
           <t>PCM-scoped only. No Doc-Draw-Quant-Cost-Schedule traversal, no lineage or downstream-impact APIs.</t>
         </is>
       </c>
-      <c r="F43" s="18" t="inlineStr">
+      <c r="F44" s="18" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
       </c>
-      <c r="G43" s="6" t="inlineStr">
+      <c r="G44" s="6" t="inlineStr">
         <is>
           <t>XL</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A4:G43"/>
+  <autoFilter ref="A4:G44"/>
   <mergeCells count="2">
     <mergeCell ref="A2:G2"/>
     <mergeCell ref="A1:G1"/>
@@ -2683,7 +2722,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F22"/>
+  <dimension ref="A1:F20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -2972,22 +3011,22 @@
       </c>
       <c r="B12" s="5" t="inlineStr">
         <is>
-          <t>Per-attempt usage ledger</t>
-        </is>
-      </c>
-      <c r="C12" s="17" t="inlineStr">
-        <is>
-          <t>Missing</t>
+          <t>Retrieval / RAG</t>
+        </is>
+      </c>
+      <c r="C12" s="18" t="inlineStr">
+        <is>
+          <t>Partial</t>
         </is>
       </c>
       <c r="D12" s="5" t="inlineStr">
         <is>
-          <t>A retry overwrites the previous attempt tokens, so failed-attempt spend is invisible and AI cost is under-counted today.</t>
+          <t>Wired for DocLogix only. No embeddings generated, and the AI worker does not call it yet - so agents still answer from the envelope.</t>
         </is>
       </c>
       <c r="E12" s="6" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>M</t>
         </is>
       </c>
       <c r="F12" s="17" t="inlineStr">
@@ -3004,22 +3043,22 @@
       </c>
       <c r="B13" s="5" t="inlineStr">
         <is>
-          <t>Tenant AI policy and data sensitivity</t>
-        </is>
-      </c>
-      <c r="C13" s="17" t="inlineStr">
-        <is>
-          <t>Missing</t>
+          <t>AI cost reporting</t>
+        </is>
+      </c>
+      <c r="C13" s="18" t="inlineStr">
+        <is>
+          <t>Partial</t>
         </is>
       </c>
       <c r="D13" s="5" t="inlineStr">
         <is>
-          <t>Blocks Preckon Private AI and Sovereign AI as sellable products.</t>
+          <t>Built on under-counted data until the per-attempt ledger exists.</t>
         </is>
       </c>
       <c r="E13" s="6" t="inlineStr">
         <is>
-          <t>L</t>
+          <t>S</t>
         </is>
       </c>
       <c r="F13" s="17" t="inlineStr">
@@ -3036,22 +3075,22 @@
       </c>
       <c r="B14" s="5" t="inlineStr">
         <is>
-          <t>Retrieval / RAG</t>
-        </is>
-      </c>
-      <c r="C14" s="18" t="inlineStr">
-        <is>
-          <t>Partial</t>
+          <t>CI running the test suite</t>
+        </is>
+      </c>
+      <c r="C14" s="17" t="inlineStr">
+        <is>
+          <t>Missing</t>
         </is>
       </c>
       <c r="D14" s="5" t="inlineStr">
         <is>
-          <t>Wired for DocLogix only. No embeddings generated, and the AI worker does not call it yet - so agents still answer from the envelope.</t>
+          <t>426 tests and six quality gates run only on a developer machine.</t>
         </is>
       </c>
       <c r="E14" s="6" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>S</t>
         </is>
       </c>
       <c r="F14" s="17" t="inlineStr">
@@ -3068,22 +3107,22 @@
       </c>
       <c r="B15" s="5" t="inlineStr">
         <is>
-          <t>AI cost reporting</t>
-        </is>
-      </c>
-      <c r="C15" s="18" t="inlineStr">
-        <is>
-          <t>Partial</t>
+          <t>Automated backup and tested restore</t>
+        </is>
+      </c>
+      <c r="C15" s="17" t="inlineStr">
+        <is>
+          <t>Missing</t>
         </is>
       </c>
       <c r="D15" s="5" t="inlineStr">
         <is>
-          <t>Built on under-counted data until the per-attempt ledger exists.</t>
+          <t>An untested restore is not a backup.</t>
         </is>
       </c>
       <c r="E15" s="6" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>M</t>
         </is>
       </c>
       <c r="F15" s="17" t="inlineStr">
@@ -3100,7 +3139,7 @@
       </c>
       <c r="B16" s="5" t="inlineStr">
         <is>
-          <t>CI running the test suite</t>
+          <t>Staging environment</t>
         </is>
       </c>
       <c r="C16" s="17" t="inlineStr">
@@ -3110,12 +3149,12 @@
       </c>
       <c r="D16" s="5" t="inlineStr">
         <is>
-          <t>426 tests and six quality gates run only on a developer machine.</t>
+          <t>Changes are currently validated in production.</t>
         </is>
       </c>
       <c r="E16" s="6" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>M</t>
         </is>
       </c>
       <c r="F16" s="17" t="inlineStr">
@@ -3132,7 +3171,7 @@
       </c>
       <c r="B17" s="5" t="inlineStr">
         <is>
-          <t>Automated backup and tested restore</t>
+          <t>Branch protection and PR review</t>
         </is>
       </c>
       <c r="C17" s="17" t="inlineStr">
@@ -3142,12 +3181,12 @@
       </c>
       <c r="D17" s="5" t="inlineStr">
         <is>
-          <t>An untested restore is not a backup.</t>
+          <t>No review gate on production code.</t>
         </is>
       </c>
       <c r="E17" s="6" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>S</t>
         </is>
       </c>
       <c r="F17" s="17" t="inlineStr">
@@ -3164,7 +3203,7 @@
       </c>
       <c r="B18" s="5" t="inlineStr">
         <is>
-          <t>Staging environment</t>
+          <t>Encryption at rest and key management</t>
         </is>
       </c>
       <c r="C18" s="17" t="inlineStr">
@@ -3174,12 +3213,12 @@
       </c>
       <c r="D18" s="5" t="inlineStr">
         <is>
-          <t>Changes are currently validated in production.</t>
+          <t>Named in Complete Platform section 15.</t>
         </is>
       </c>
       <c r="E18" s="6" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>L</t>
         </is>
       </c>
       <c r="F18" s="17" t="inlineStr">
@@ -3196,7 +3235,7 @@
       </c>
       <c r="B19" s="5" t="inlineStr">
         <is>
-          <t>Branch protection and PR review</t>
+          <t>Credential rotation</t>
         </is>
       </c>
       <c r="C19" s="17" t="inlineStr">
@@ -3206,7 +3245,7 @@
       </c>
       <c r="D19" s="5" t="inlineStr">
         <is>
-          <t>No review gate on production code.</t>
+          <t>Rotate everything ever committed; confirm the production DB password is not the default.</t>
         </is>
       </c>
       <c r="E19" s="6" t="inlineStr">
@@ -3228,22 +3267,22 @@
       </c>
       <c r="B20" s="5" t="inlineStr">
         <is>
-          <t>Encryption at rest and key management</t>
-        </is>
-      </c>
-      <c r="C20" s="17" t="inlineStr">
-        <is>
-          <t>Missing</t>
+          <t>Port hardening</t>
+        </is>
+      </c>
+      <c r="C20" s="18" t="inlineStr">
+        <is>
+          <t>Partial</t>
         </is>
       </c>
       <c r="D20" s="5" t="inlineStr">
         <is>
-          <t>Named in Complete Platform section 15.</t>
+          <t>3307 (MySQL), 11434 (Ollama, unauthenticated) and 5000 bind 0.0.0.0; only the provider firewall stops them.</t>
         </is>
       </c>
       <c r="E20" s="6" t="inlineStr">
         <is>
-          <t>L</t>
+          <t>S</t>
         </is>
       </c>
       <c r="F20" s="17" t="inlineStr">
@@ -3252,72 +3291,8 @@
         </is>
       </c>
     </row>
-    <row r="21">
-      <c r="A21" s="15" t="inlineStr">
-        <is>
-          <t>Platform / Core</t>
-        </is>
-      </c>
-      <c r="B21" s="5" t="inlineStr">
-        <is>
-          <t>Credential rotation</t>
-        </is>
-      </c>
-      <c r="C21" s="17" t="inlineStr">
-        <is>
-          <t>Missing</t>
-        </is>
-      </c>
-      <c r="D21" s="5" t="inlineStr">
-        <is>
-          <t>Rotate everything ever committed; confirm the production DB password is not the default.</t>
-        </is>
-      </c>
-      <c r="E21" s="6" t="inlineStr">
-        <is>
-          <t>S</t>
-        </is>
-      </c>
-      <c r="F21" s="17" t="inlineStr">
-        <is>
-          <t>P0</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="15" t="inlineStr">
-        <is>
-          <t>Platform / Core</t>
-        </is>
-      </c>
-      <c r="B22" s="5" t="inlineStr">
-        <is>
-          <t>Port hardening</t>
-        </is>
-      </c>
-      <c r="C22" s="18" t="inlineStr">
-        <is>
-          <t>Partial</t>
-        </is>
-      </c>
-      <c r="D22" s="5" t="inlineStr">
-        <is>
-          <t>3307 (MySQL), 11434 (Ollama, unauthenticated) and 5000 bind 0.0.0.0; only the provider firewall stops them.</t>
-        </is>
-      </c>
-      <c r="E22" s="6" t="inlineStr">
-        <is>
-          <t>S</t>
-        </is>
-      </c>
-      <c r="F22" s="17" t="inlineStr">
-        <is>
-          <t>P0</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A4:F22"/>
+  <autoFilter ref="A4:F20"/>
   <mergeCells count="2">
     <mergeCell ref="A2:F2"/>
     <mergeCell ref="A1:F1"/>
@@ -3447,7 +3422,7 @@
       </c>
       <c r="B9" s="20" t="inlineStr">
         <is>
-          <t>71</t>
+          <t>77</t>
         </is>
       </c>
       <c r="C9" s="5" t="inlineStr">
@@ -3464,7 +3439,7 @@
       </c>
       <c r="B10" s="20" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>21</t>
         </is>
       </c>
       <c r="C10" s="5" t="inlineStr">
@@ -3515,12 +3490,12 @@
       </c>
       <c r="B13" s="20" t="inlineStr">
         <is>
-          <t>632 passing</t>
+          <t>753 passing</t>
         </is>
       </c>
       <c r="C13" s="5" t="inlineStr">
         <is>
-          <t>29 files. Was 426 on 19 Aug; DocLogix added 206. One pre-existing failure needs Docker MySQL on 3308.</t>
+          <t>33 files. Was 426 on 19 Aug. DocLogix added 206, AI governance and upload safety a further 121. One pre-existing failure needs Docker MySQL on 3308.</t>
         </is>
       </c>
     </row>
@@ -3532,12 +3507,12 @@
       </c>
       <c r="B14" s="20" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>15</t>
         </is>
       </c>
       <c r="C14" s="5" t="inlineStr">
         <is>
-          <t>cpm, pcm/measure, boq/reconcile, cad/compare, cad/impact, standards, validate, doc/numbering, doc/revision, doc/compare, doc/retrieval</t>
+          <t>cpm, pcm/measure, boq/reconcile, cad/compare, cad/impact, standards, validate, doc/numbering, doc/revision, doc/compare, doc/retrieval, ai/policy, ai/budget, ai/cache, upload-safety</t>
         </is>
       </c>
     </row>
@@ -3600,12 +3575,12 @@
       </c>
       <c r="B18" s="20" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>8</t>
         </is>
       </c>
       <c r="C18" s="5" t="inlineStr">
         <is>
-          <t>50 are specified across three blueprints</t>
+          <t>Of ~50 specified. Cover the three-way stack conflict, queue choice, AI authority, model aliases, tenant policy, usage ledger, cache safety and tenant isolation.</t>
         </is>
       </c>
     </row>
@@ -3650,6 +3625,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4" ht="34" customHeight="1">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -4395,6 +4371,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4" ht="34" customHeight="1">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -5029,6 +5006,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4" ht="34" customHeight="1">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -5700,6 +5678,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4" ht="34" customHeight="1">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -6186,6 +6165,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4" ht="34" customHeight="1">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -6561,6 +6541,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4" ht="34" customHeight="1">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -7195,6 +7176,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4" ht="34" customHeight="1">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -7496,6 +7478,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4" ht="34" customHeight="1">
       <c r="A4" s="3" t="inlineStr">
         <is>

</xml_diff>